<commit_message>
feat: complete Task 3.4 Program Loader implementation
- Added ClearCodeSegment to reset 00h-1Fh memory range safely.
- Added UI methods to read and write the program source cell (K25).
- Implemented ParseHexProgram, LoadProgramFromBytes, LoadProgram, and LoadDemoProgram in main.js.
- Ensured all loader memory writes route through the system Bus.
- Updated README documentation for the program source cell and loader state.
</commit_message>
<xml_diff>
--- a/simulator.xlsx
+++ b/simulator.xlsx
@@ -16,11 +16,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t xml:space="preserve">8-BIT VON NEUMANN CPU SIMULATOR</t>
   </si>
   <si>
+    <t>i</t>
+  </si>
+  <si>
     <t>Register</t>
   </si>
   <si>
@@ -36,6 +39,9 @@
     <t>PC</t>
   </si>
   <si>
+    <t>0B</t>
+  </si>
+  <si>
     <t>RAM</t>
   </si>
   <si>
@@ -66,33 +72,24 @@
     <t>MAR</t>
   </si>
   <si>
+    <t>0A</t>
+  </si>
+  <si>
     <t xml:space="preserve">Code Segment</t>
   </si>
   <si>
     <t>00h</t>
   </si>
   <si>
-    <t>0F</t>
-  </si>
-  <si>
     <t>MDR</t>
   </si>
   <si>
-    <t>1F</t>
-  </si>
-  <si>
     <t>10h</t>
   </si>
   <si>
-    <t>1A</t>
-  </si>
-  <si>
     <t>AX</t>
   </si>
   <si>
-    <t>2C</t>
-  </si>
-  <si>
     <t xml:space="preserve">Reserved Area</t>
   </si>
   <si>
@@ -102,9 +99,6 @@
     <t>BX</t>
   </si>
   <si>
-    <t>AB</t>
-  </si>
-  <si>
     <t>30h</t>
   </si>
   <si>
@@ -181,9 +175,6 @@
   </si>
   <si>
     <t>F0h</t>
-  </si>
-  <si>
-    <t>FF</t>
   </si>
   <si>
     <t xml:space="preserve">Delay (ms):</t>
@@ -1062,35 +1053,40 @@
       <c r="Y3" s="1"/>
       <c r="Z3" s="1"/>
     </row>
+    <row r="4" ht="14.25">
+      <c r="O4" t="s">
+        <v>1</v>
+      </c>
+    </row>
     <row r="5" ht="14.25">
       <c r="B5" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" ht="14.25">
       <c r="B6" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="4">
-        <v>15</v>
+        <v>6</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="D6" s="4">
-        <v>10101</v>
+        <v>1011</v>
       </c>
       <c r="E6" s="4">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
@@ -1111,19 +1107,19 @@
     </row>
     <row r="7" ht="14.25">
       <c r="B7" s="3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C7" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" s="4">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E7" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K7" s="4">
         <v>0</v>
@@ -1156,45 +1152,45 @@
         <v>9</v>
       </c>
       <c r="U7" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="V7" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="W7" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="X7" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="Y7" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="Z7" s="4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" ht="14.25">
       <c r="B8" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="4">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>18</v>
       </c>
       <c r="D8" s="4">
-        <v>0</v>
+        <v>1010</v>
       </c>
       <c r="E8" s="4">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K8" s="7" t="s">
-        <v>18</v>
+        <v>20</v>
+      </c>
+      <c r="K8" s="7">
+        <v>0</v>
       </c>
       <c r="L8" s="7">
         <v>0</v>
@@ -1224,7 +1220,7 @@
         <v>0</v>
       </c>
       <c r="U8" s="7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V8" s="7">
         <v>0</v>
@@ -1244,20 +1240,20 @@
     </row>
     <row r="9" ht="14.25">
       <c r="B9" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="C9" s="4">
+        <v>2</v>
       </c>
       <c r="D9" s="4">
-        <v>11111</v>
+        <v>10</v>
       </c>
       <c r="E9" s="4">
-        <v>31</v>
+        <v>2</v>
       </c>
       <c r="I9" s="6"/>
       <c r="J9" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K9" s="7">
         <v>0</v>
@@ -1289,8 +1285,8 @@
       <c r="T9" s="7">
         <v>0</v>
       </c>
-      <c r="U9" s="7" t="s">
-        <v>22</v>
+      <c r="U9" s="7">
+        <v>0</v>
       </c>
       <c r="V9" s="7">
         <v>0</v>
@@ -1312,20 +1308,20 @@
       <c r="B10" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="4">
+        <v>0</v>
+      </c>
+      <c r="D10" s="4">
+        <v>0</v>
+      </c>
+      <c r="E10" s="4">
+        <v>0</v>
+      </c>
+      <c r="I10" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="4">
-        <v>101100</v>
-      </c>
-      <c r="E10" s="4">
-        <v>44</v>
-      </c>
-      <c r="I10" s="8" t="s">
+      <c r="J10" s="4" t="s">
         <v>25</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>26</v>
       </c>
       <c r="K10" s="9">
         <v>0</v>
@@ -1378,20 +1374,20 @@
     </row>
     <row r="11" ht="14.25">
       <c r="B11" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>28</v>
+        <v>26</v>
+      </c>
+      <c r="C11" s="4">
+        <v>0</v>
       </c>
       <c r="D11" s="4">
-        <v>10101011</v>
+        <v>0</v>
       </c>
       <c r="E11" s="4">
-        <v>171</v>
+        <v>0</v>
       </c>
       <c r="I11" s="10"/>
       <c r="J11" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K11" s="9">
         <v>0</v>
@@ -1445,7 +1441,7 @@
     <row r="12" ht="14.25">
       <c r="I12" s="10"/>
       <c r="J12" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K12" s="9">
         <v>0</v>
@@ -1498,14 +1494,14 @@
     </row>
     <row r="13" ht="14.25">
       <c r="B13" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
       <c r="I13" s="10"/>
       <c r="J13" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K13" s="9">
         <v>0</v>
@@ -1558,16 +1554,16 @@
     </row>
     <row r="14" ht="14.25">
       <c r="B14" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C14" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="13"/>
       <c r="I14" s="10"/>
       <c r="J14" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="K14" s="9">
         <v>0</v>
@@ -1620,7 +1616,7 @@
     </row>
     <row r="15" ht="14.25">
       <c r="B15" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C15" s="11">
         <v>0</v>
@@ -1629,7 +1625,7 @@
       <c r="E15" s="13"/>
       <c r="I15" s="14"/>
       <c r="J15" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="K15" s="9">
         <v>0</v>
@@ -1682,18 +1678,18 @@
     </row>
     <row r="16" ht="14.25">
       <c r="B16" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C16" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="13"/>
       <c r="I16" s="8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="K16" s="15">
         <v>0</v>
@@ -1747,7 +1743,7 @@
     <row r="17" ht="14.25">
       <c r="I17" s="10"/>
       <c r="J17" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="K17" s="15">
         <v>0</v>
@@ -1800,16 +1796,16 @@
     </row>
     <row r="18" ht="14.25">
       <c r="B18" s="16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="I18" s="10"/>
       <c r="J18" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="K18" s="15">
         <v>0</v>
@@ -1862,7 +1858,7 @@
     </row>
     <row r="19" ht="14.25">
       <c r="B19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C19" s="17">
         <v>0</v>
@@ -1871,7 +1867,7 @@
       <c r="E19" s="17"/>
       <c r="I19" s="10"/>
       <c r="J19" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K19" s="15">
         <v>0</v>
@@ -1925,7 +1921,7 @@
     <row r="20" ht="14.25">
       <c r="I20" s="10"/>
       <c r="J20" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="K20" s="15">
         <v>0</v>
@@ -1978,16 +1974,16 @@
     </row>
     <row r="21" ht="14.25">
       <c r="B21" s="18" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C21" s="18"/>
       <c r="D21" s="18" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E21" s="19"/>
       <c r="I21" s="10"/>
       <c r="J21" s="4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="K21" s="15">
         <v>0</v>
@@ -2040,16 +2036,16 @@
     </row>
     <row r="22" ht="14.25">
       <c r="B22" s="18" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C22" s="18"/>
       <c r="D22" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E22" s="18"/>
       <c r="I22" s="10"/>
       <c r="J22" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="K22" s="15">
         <v>0</v>
@@ -2102,14 +2098,14 @@
     </row>
     <row r="23" ht="14.25">
       <c r="B23" s="18" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C23" s="18"/>
       <c r="D23" s="18"/>
       <c r="E23" s="18"/>
       <c r="I23" s="14"/>
       <c r="J23" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="K23" s="15">
         <v>0</v>
@@ -2156,13 +2152,13 @@
       <c r="Y23" s="15">
         <v>0</v>
       </c>
-      <c r="Z23" s="15" t="s">
-        <v>55</v>
+      <c r="Z23" s="15">
+        <v>0</v>
       </c>
     </row>
     <row r="24" ht="14.25">
       <c r="B24" s="17" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C24" s="17">
         <v>500</v>
@@ -2172,7 +2168,7 @@
     </row>
     <row r="26" ht="14.25">
       <c r="B26" s="20" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C26" s="20"/>
       <c r="D26" s="20"/>
@@ -2201,34 +2197,34 @@
     </row>
     <row r="27" ht="14.25">
       <c r="B27" s="21" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E27" s="21" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F27" s="21" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G27" s="21" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H27" s="21" t="s">
         <v>23</v>
       </c>
       <c r="I27" s="21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J27" s="21" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="K27" s="21" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="L27" s="21"/>
       <c r="M27" s="21"/>

</xml_diff>